<commit_message>
time lab 2 W
</commit_message>
<xml_diff>
--- a/tl02/tl02microcode.xlsx
+++ b/tl02/tl02microcode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26611"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26501"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/avagavin/Documents/Spring 2023/CS 2110/TL2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huan\Documents\GT\Summer 2023\CS_2110\tl02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE3115B8-D17B-4FF7-B769-6683F52542F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A3AFA7-B15C-450D-B810-55FB44085633}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1840" yWindow="500" windowWidth="25320" windowHeight="15580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="microcode" sheetId="1" r:id="rId1"/>
@@ -1305,14 +1305,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BW66"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11.08203125" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="30" width="4.625" customWidth="1"/>
-    <col min="31" max="31" width="2.625" customWidth="1"/>
+    <col min="2" max="30" width="4.58203125" customWidth="1"/>
+    <col min="31" max="31" width="2.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:75" ht="90">
+    <row r="1" spans="1:75" ht="88">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="21" t="s">
@@ -1402,7 +1402,7 @@
       <c r="AF1" s="3"/>
       <c r="AG1" s="3"/>
     </row>
-    <row r="2" spans="1:75" ht="15.75">
+    <row r="2" spans="1:75">
       <c r="A2" s="4"/>
       <c r="B2" s="5"/>
       <c r="C2" s="23"/>
@@ -1437,7 +1437,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:75" ht="32.1" customHeight="1">
+    <row r="3" spans="1:75" ht="32.15" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>23</v>
       </c>
@@ -1476,32 +1476,72 @@
         <v>24</v>
       </c>
       <c r="B4" s="8"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
-      <c r="M4" s="43"/>
-      <c r="N4" s="54"/>
+      <c r="C4" s="23">
+        <v>0</v>
+      </c>
+      <c r="D4" s="23">
+        <v>0</v>
+      </c>
+      <c r="E4" s="23">
+        <v>0</v>
+      </c>
+      <c r="F4" s="23">
+        <v>1</v>
+      </c>
+      <c r="G4" s="23">
+        <v>1</v>
+      </c>
+      <c r="H4" s="23">
+        <v>0</v>
+      </c>
+      <c r="I4" s="34">
+        <v>0</v>
+      </c>
+      <c r="J4" s="34">
+        <v>0</v>
+      </c>
+      <c r="K4" s="34">
+        <v>0</v>
+      </c>
+      <c r="L4" s="34">
+        <v>1</v>
+      </c>
+      <c r="M4" s="43">
+        <v>0</v>
+      </c>
+      <c r="N4" s="54">
+        <v>0</v>
+      </c>
       <c r="O4" s="72">
         <v>0</v>
       </c>
       <c r="P4" s="72">
         <v>0</v>
       </c>
-      <c r="Q4" s="55"/>
-      <c r="R4" s="43"/>
-      <c r="S4" s="54"/>
-      <c r="T4" s="55"/>
-      <c r="U4" s="43"/>
-      <c r="V4" s="54"/>
-      <c r="W4" s="63"/>
-      <c r="X4" s="63"/>
+      <c r="Q4" s="55">
+        <v>1</v>
+      </c>
+      <c r="R4" s="43">
+        <v>1</v>
+      </c>
+      <c r="S4" s="54">
+        <v>0</v>
+      </c>
+      <c r="T4" s="55">
+        <v>1</v>
+      </c>
+      <c r="U4" s="43">
+        <v>1</v>
+      </c>
+      <c r="V4" s="54">
+        <v>1</v>
+      </c>
+      <c r="W4" s="63">
+        <v>0</v>
+      </c>
+      <c r="X4" s="63">
+        <v>0</v>
+      </c>
       <c r="Y4" s="87">
         <v>0</v>
       </c>
@@ -1522,12 +1562,12 @@
       </c>
       <c r="AH4" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C4:F4), 1), BIN2HEX(_xlfn.CONCAT(G4:N4), 2), BIN2HEX(_xlfn.CONCAT(O4:V4), 2), BIN2HEX(_xlfn.CONCAT(W4:AD4), 2) )</f>
-        <v>0000008</v>
+        <v>1843708</v>
       </c>
       <c r="BQ4" s="3"/>
       <c r="BR4" s="3"/>
     </row>
-    <row r="5" spans="1:75" ht="30.95">
+    <row r="5" spans="1:75" ht="31">
       <c r="A5" s="11" t="s">
         <v>25</v>
       </c>
@@ -1596,32 +1636,72 @@
       <c r="A7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="38"/>
-      <c r="J7" s="38"/>
-      <c r="K7" s="38"/>
-      <c r="L7" s="38"/>
-      <c r="M7" s="49"/>
-      <c r="N7" s="48"/>
+      <c r="C7" s="25">
+        <v>1</v>
+      </c>
+      <c r="D7" s="27">
+        <v>0</v>
+      </c>
+      <c r="E7" s="27">
+        <v>0</v>
+      </c>
+      <c r="F7" s="27">
+        <v>0</v>
+      </c>
+      <c r="G7" s="27">
+        <v>0</v>
+      </c>
+      <c r="H7" s="27">
+        <v>0</v>
+      </c>
+      <c r="I7" s="38">
+        <v>0</v>
+      </c>
+      <c r="J7" s="38">
+        <v>0</v>
+      </c>
+      <c r="K7" s="38">
+        <v>0</v>
+      </c>
+      <c r="L7" s="38">
+        <v>1</v>
+      </c>
+      <c r="M7" s="49">
+        <v>0</v>
+      </c>
+      <c r="N7" s="48">
+        <v>0</v>
+      </c>
       <c r="O7" s="74">
         <v>0</v>
       </c>
       <c r="P7" s="74">
         <v>0</v>
       </c>
-      <c r="Q7" s="48"/>
-      <c r="R7" s="49"/>
-      <c r="S7" s="48"/>
-      <c r="T7" s="48"/>
-      <c r="U7" s="49"/>
-      <c r="V7" s="48"/>
-      <c r="W7" s="65"/>
-      <c r="X7" s="65"/>
+      <c r="Q7" s="48">
+        <v>0</v>
+      </c>
+      <c r="R7" s="49">
+        <v>1</v>
+      </c>
+      <c r="S7" s="48">
+        <v>0</v>
+      </c>
+      <c r="T7" s="48">
+        <v>1</v>
+      </c>
+      <c r="U7" s="49">
+        <v>0</v>
+      </c>
+      <c r="V7" s="48">
+        <v>0</v>
+      </c>
+      <c r="W7" s="65">
+        <v>0</v>
+      </c>
+      <c r="X7" s="65">
+        <v>0</v>
+      </c>
       <c r="Y7" s="77">
         <v>0</v>
       </c>
@@ -1642,39 +1722,79 @@
       </c>
       <c r="AH7" t="str">
         <f t="shared" ref="AH7:AH8" si="0">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C7:F7), 1), BIN2HEX(_xlfn.CONCAT(G7:N7), 2), BIN2HEX(_xlfn.CONCAT(O7:V7), 2), BIN2HEX(_xlfn.CONCAT(W7:AD7), 2) )</f>
-        <v>0000017</v>
+        <v>8041417</v>
       </c>
     </row>
     <row r="8" spans="1:75">
       <c r="A8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="38"/>
-      <c r="J8" s="38"/>
-      <c r="K8" s="38"/>
-      <c r="L8" s="38"/>
-      <c r="M8" s="49"/>
-      <c r="N8" s="48"/>
+      <c r="C8" s="25">
+        <v>0</v>
+      </c>
+      <c r="D8" s="27">
+        <v>1</v>
+      </c>
+      <c r="E8" s="27">
+        <v>0</v>
+      </c>
+      <c r="F8" s="27">
+        <v>0</v>
+      </c>
+      <c r="G8" s="27">
+        <v>0</v>
+      </c>
+      <c r="H8" s="27">
+        <v>0</v>
+      </c>
+      <c r="I8" s="38">
+        <v>0</v>
+      </c>
+      <c r="J8" s="38">
+        <v>0</v>
+      </c>
+      <c r="K8" s="38">
+        <v>0</v>
+      </c>
+      <c r="L8" s="38">
+        <v>0</v>
+      </c>
+      <c r="M8" s="49">
+        <v>0</v>
+      </c>
+      <c r="N8" s="48">
+        <v>0</v>
+      </c>
       <c r="O8" s="74">
         <v>0</v>
       </c>
       <c r="P8" s="74">
         <v>0</v>
       </c>
-      <c r="Q8" s="48"/>
-      <c r="R8" s="49"/>
-      <c r="S8" s="48"/>
-      <c r="T8" s="48"/>
-      <c r="U8" s="49"/>
-      <c r="V8" s="48"/>
-      <c r="W8" s="65"/>
-      <c r="X8" s="65"/>
+      <c r="Q8" s="48">
+        <v>0</v>
+      </c>
+      <c r="R8" s="49">
+        <v>0</v>
+      </c>
+      <c r="S8" s="48">
+        <v>0</v>
+      </c>
+      <c r="T8" s="48">
+        <v>0</v>
+      </c>
+      <c r="U8" s="49">
+        <v>0</v>
+      </c>
+      <c r="V8" s="48">
+        <v>0</v>
+      </c>
+      <c r="W8" s="65">
+        <v>1</v>
+      </c>
+      <c r="X8" s="65">
+        <v>0</v>
+      </c>
       <c r="Y8" s="77">
         <v>1</v>
       </c>
@@ -1695,7 +1815,7 @@
       </c>
       <c r="AH8" t="str">
         <f t="shared" si="0"/>
-        <v>0000027</v>
+        <v>40000A7</v>
       </c>
     </row>
     <row r="9" spans="1:75">
@@ -1703,32 +1823,72 @@
         <v>28</v>
       </c>
       <c r="B9" s="8"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="I9" s="39"/>
-      <c r="J9" s="39"/>
-      <c r="K9" s="39"/>
-      <c r="L9" s="39"/>
-      <c r="M9" s="58"/>
-      <c r="N9" s="54"/>
+      <c r="C9" s="28">
+        <v>0</v>
+      </c>
+      <c r="D9" s="29">
+        <v>0</v>
+      </c>
+      <c r="E9" s="29">
+        <v>0</v>
+      </c>
+      <c r="F9" s="29">
+        <v>0</v>
+      </c>
+      <c r="G9" s="29">
+        <v>0</v>
+      </c>
+      <c r="H9" s="29">
+        <v>1</v>
+      </c>
+      <c r="I9" s="39">
+        <v>0</v>
+      </c>
+      <c r="J9" s="39">
+        <v>1</v>
+      </c>
+      <c r="K9" s="39">
+        <v>0</v>
+      </c>
+      <c r="L9" s="39">
+        <v>0</v>
+      </c>
+      <c r="M9" s="58">
+        <v>1</v>
+      </c>
+      <c r="N9" s="54">
+        <v>0</v>
+      </c>
       <c r="O9" s="75">
         <v>0</v>
       </c>
       <c r="P9" s="74">
         <v>0</v>
       </c>
-      <c r="Q9" s="54"/>
-      <c r="R9" s="58"/>
-      <c r="S9" s="54"/>
-      <c r="T9" s="54"/>
-      <c r="U9" s="58"/>
-      <c r="V9" s="54"/>
-      <c r="W9" s="66"/>
-      <c r="X9" s="66"/>
+      <c r="Q9" s="54">
+        <v>0</v>
+      </c>
+      <c r="R9" s="58">
+        <v>0</v>
+      </c>
+      <c r="S9" s="54">
+        <v>0</v>
+      </c>
+      <c r="T9" s="54">
+        <v>0</v>
+      </c>
+      <c r="U9" s="58">
+        <v>0</v>
+      </c>
+      <c r="V9" s="54">
+        <v>0</v>
+      </c>
+      <c r="W9" s="66">
+        <v>0</v>
+      </c>
+      <c r="X9" s="66">
+        <v>0</v>
+      </c>
       <c r="Y9" s="88">
         <v>0</v>
       </c>
@@ -1749,10 +1909,10 @@
       </c>
       <c r="AH9" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C9:F9), 1), BIN2HEX(_xlfn.CONCAT(G9:N9), 2), BIN2HEX(_xlfn.CONCAT(O9:V9), 2), BIN2HEX(_xlfn.CONCAT(W9:AD9), 2) )</f>
-        <v>0000008</v>
-      </c>
-    </row>
-    <row r="10" spans="1:75" ht="32.1" customHeight="1">
+        <v>0520008</v>
+      </c>
+    </row>
+    <row r="10" spans="1:75" ht="32.15" customHeight="1">
       <c r="A10" s="19" t="s">
         <v>29</v>
       </c>
@@ -1822,32 +1982,72 @@
         <v>30</v>
       </c>
       <c r="B12" s="8"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="29"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39"/>
-      <c r="M12" s="58"/>
-      <c r="N12" s="54"/>
+      <c r="C12" s="28">
+        <v>0</v>
+      </c>
+      <c r="D12" s="29">
+        <v>0</v>
+      </c>
+      <c r="E12" s="29">
+        <v>0</v>
+      </c>
+      <c r="F12" s="29">
+        <v>0</v>
+      </c>
+      <c r="G12" s="29">
+        <v>0</v>
+      </c>
+      <c r="H12" s="29">
+        <v>1</v>
+      </c>
+      <c r="I12" s="39">
+        <v>0</v>
+      </c>
+      <c r="J12" s="39">
+        <v>0</v>
+      </c>
+      <c r="K12" s="39">
+        <v>0</v>
+      </c>
+      <c r="L12" s="39">
+        <v>1</v>
+      </c>
+      <c r="M12" s="58">
+        <v>1</v>
+      </c>
+      <c r="N12" s="54">
+        <v>0</v>
+      </c>
       <c r="O12" s="75">
         <v>0</v>
       </c>
       <c r="P12" s="72">
         <v>0</v>
       </c>
-      <c r="Q12" s="54"/>
-      <c r="R12" s="58"/>
-      <c r="S12" s="54"/>
-      <c r="T12" s="54"/>
-      <c r="U12" s="58"/>
-      <c r="V12" s="54"/>
-      <c r="W12" s="66"/>
-      <c r="X12" s="66"/>
+      <c r="Q12" s="54">
+        <v>0</v>
+      </c>
+      <c r="R12" s="58">
+        <v>1</v>
+      </c>
+      <c r="S12" s="54">
+        <v>1</v>
+      </c>
+      <c r="T12" s="54">
+        <v>1</v>
+      </c>
+      <c r="U12" s="58">
+        <v>0</v>
+      </c>
+      <c r="V12" s="54">
+        <v>0</v>
+      </c>
+      <c r="W12" s="66">
+        <v>0</v>
+      </c>
+      <c r="X12" s="66">
+        <v>0</v>
+      </c>
       <c r="Y12" s="88">
         <v>0</v>
       </c>
@@ -1868,10 +2068,10 @@
       </c>
       <c r="AH12" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C12:F12), 1), BIN2HEX(_xlfn.CONCAT(G12:N12), 2), BIN2HEX(_xlfn.CONCAT(O12:V12), 2), BIN2HEX(_xlfn.CONCAT(W12:AD12), 2) )</f>
-        <v>0000008</v>
-      </c>
-    </row>
-    <row r="13" spans="1:75" ht="32.1" customHeight="1">
+        <v>0461C08</v>
+      </c>
+    </row>
+    <row r="13" spans="1:75" ht="32.15" customHeight="1">
       <c r="A13" s="9" t="s">
         <v>31</v>
       </c>
@@ -1905,7 +2105,7 @@
       <c r="AC13" s="77"/>
       <c r="AD13" s="83"/>
     </row>
-    <row r="14" spans="1:75" ht="16.350000000000001" customHeight="1">
+    <row r="14" spans="1:75" ht="16.399999999999999" customHeight="1">
       <c r="A14" s="7"/>
       <c r="C14" s="30"/>
       <c r="D14" s="31"/>
@@ -1940,32 +2140,72 @@
       <c r="A15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
-      <c r="I15" s="38"/>
-      <c r="J15" s="38"/>
-      <c r="K15" s="38"/>
-      <c r="L15" s="38"/>
-      <c r="M15" s="49"/>
-      <c r="N15" s="48"/>
+      <c r="C15" s="30">
+        <v>0</v>
+      </c>
+      <c r="D15" s="31">
+        <v>0</v>
+      </c>
+      <c r="E15" s="31">
+        <v>0</v>
+      </c>
+      <c r="F15" s="31">
+        <v>1</v>
+      </c>
+      <c r="G15" s="31">
+        <v>1</v>
+      </c>
+      <c r="H15" s="31">
+        <v>0</v>
+      </c>
+      <c r="I15" s="38">
+        <v>0</v>
+      </c>
+      <c r="J15" s="38">
+        <v>0</v>
+      </c>
+      <c r="K15" s="38">
+        <v>1</v>
+      </c>
+      <c r="L15" s="38">
+        <v>0</v>
+      </c>
+      <c r="M15" s="49">
+        <v>0</v>
+      </c>
+      <c r="N15" s="48">
+        <v>0</v>
+      </c>
       <c r="O15" s="74">
         <v>0</v>
       </c>
       <c r="P15" s="74">
         <v>1</v>
       </c>
-      <c r="Q15" s="48"/>
-      <c r="R15" s="49"/>
-      <c r="S15" s="48"/>
-      <c r="T15" s="48"/>
-      <c r="U15" s="49"/>
-      <c r="V15" s="48"/>
-      <c r="W15" s="65"/>
-      <c r="X15" s="65"/>
+      <c r="Q15" s="48">
+        <v>0</v>
+      </c>
+      <c r="R15" s="49">
+        <v>0</v>
+      </c>
+      <c r="S15" s="48">
+        <v>0</v>
+      </c>
+      <c r="T15" s="48">
+        <v>0</v>
+      </c>
+      <c r="U15" s="49">
+        <v>0</v>
+      </c>
+      <c r="V15" s="48">
+        <v>0</v>
+      </c>
+      <c r="W15" s="65">
+        <v>0</v>
+      </c>
+      <c r="X15" s="65">
+        <v>0</v>
+      </c>
       <c r="Y15" s="77">
         <v>0</v>
       </c>
@@ -1986,7 +2226,7 @@
       </c>
       <c r="AH15" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C15:F15), 1), BIN2HEX(_xlfn.CONCAT(G15:N15), 2), BIN2HEX(_xlfn.CONCAT(O15:V15), 2), BIN2HEX(_xlfn.CONCAT(W15:AD15), 2) )</f>
-        <v>0000116</v>
+        <v>1884016</v>
       </c>
       <c r="AL15" s="14"/>
       <c r="AM15" s="14"/>
@@ -2031,32 +2271,72 @@
       <c r="A16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="38"/>
-      <c r="J16" s="38"/>
-      <c r="K16" s="38"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="49"/>
-      <c r="N16" s="48"/>
+      <c r="C16" s="30">
+        <v>0</v>
+      </c>
+      <c r="D16" s="31">
+        <v>0</v>
+      </c>
+      <c r="E16" s="31">
+        <v>0</v>
+      </c>
+      <c r="F16" s="31">
+        <v>1</v>
+      </c>
+      <c r="G16" s="31">
+        <v>1</v>
+      </c>
+      <c r="H16" s="31">
+        <v>0</v>
+      </c>
+      <c r="I16" s="38">
+        <v>0</v>
+      </c>
+      <c r="J16" s="38">
+        <v>0</v>
+      </c>
+      <c r="K16" s="38">
+        <v>1</v>
+      </c>
+      <c r="L16" s="38">
+        <v>0</v>
+      </c>
+      <c r="M16" s="49">
+        <v>0</v>
+      </c>
+      <c r="N16" s="48">
+        <v>0</v>
+      </c>
       <c r="O16" s="74">
         <v>0</v>
       </c>
       <c r="P16" s="74">
         <v>1</v>
       </c>
-      <c r="Q16" s="48"/>
-      <c r="R16" s="49"/>
-      <c r="S16" s="48"/>
-      <c r="T16" s="48"/>
-      <c r="U16" s="49"/>
-      <c r="V16" s="48"/>
-      <c r="W16" s="65"/>
-      <c r="X16" s="65"/>
+      <c r="Q16" s="48">
+        <v>0</v>
+      </c>
+      <c r="R16" s="49">
+        <v>0</v>
+      </c>
+      <c r="S16" s="48">
+        <v>0</v>
+      </c>
+      <c r="T16" s="48">
+        <v>0</v>
+      </c>
+      <c r="U16" s="49">
+        <v>0</v>
+      </c>
+      <c r="V16" s="48">
+        <v>0</v>
+      </c>
+      <c r="W16" s="65">
+        <v>0</v>
+      </c>
+      <c r="X16" s="65">
+        <v>0</v>
+      </c>
       <c r="Y16" s="77">
         <v>1</v>
       </c>
@@ -2077,7 +2357,7 @@
       </c>
       <c r="AH16" t="str">
         <f t="shared" ref="AH16" si="1">_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C16:F16), 1), BIN2HEX(_xlfn.CONCAT(G16:N16), 2), BIN2HEX(_xlfn.CONCAT(O16:V16), 2), BIN2HEX(_xlfn.CONCAT(W16:AD16), 2) )</f>
-        <v>0000126</v>
+        <v>1884026</v>
       </c>
       <c r="AK16" s="13"/>
       <c r="AL16" s="14"/>
@@ -2124,32 +2404,72 @@
         <v>34</v>
       </c>
       <c r="B17" s="8"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="39"/>
-      <c r="L17" s="39"/>
-      <c r="M17" s="58"/>
-      <c r="N17" s="54"/>
+      <c r="C17" s="28">
+        <v>0</v>
+      </c>
+      <c r="D17" s="29">
+        <v>0</v>
+      </c>
+      <c r="E17" s="29">
+        <v>0</v>
+      </c>
+      <c r="F17" s="29">
+        <v>1</v>
+      </c>
+      <c r="G17" s="29">
+        <v>1</v>
+      </c>
+      <c r="H17" s="29">
+        <v>0</v>
+      </c>
+      <c r="I17" s="39">
+        <v>0</v>
+      </c>
+      <c r="J17" s="39">
+        <v>0</v>
+      </c>
+      <c r="K17" s="39">
+        <v>1</v>
+      </c>
+      <c r="L17" s="39">
+        <v>0</v>
+      </c>
+      <c r="M17" s="58">
+        <v>0</v>
+      </c>
+      <c r="N17" s="54">
+        <v>0</v>
+      </c>
       <c r="O17" s="75">
         <v>0</v>
       </c>
       <c r="P17" s="74">
         <v>1</v>
       </c>
-      <c r="Q17" s="54"/>
-      <c r="R17" s="58"/>
-      <c r="S17" s="54"/>
-      <c r="T17" s="54"/>
-      <c r="U17" s="58"/>
-      <c r="V17" s="54"/>
-      <c r="W17" s="66"/>
-      <c r="X17" s="66"/>
+      <c r="Q17" s="54">
+        <v>0</v>
+      </c>
+      <c r="R17" s="58">
+        <v>0</v>
+      </c>
+      <c r="S17" s="54">
+        <v>0</v>
+      </c>
+      <c r="T17" s="54">
+        <v>0</v>
+      </c>
+      <c r="U17" s="58">
+        <v>0</v>
+      </c>
+      <c r="V17" s="54">
+        <v>0</v>
+      </c>
+      <c r="W17" s="66">
+        <v>0</v>
+      </c>
+      <c r="X17" s="66">
+        <v>0</v>
+      </c>
       <c r="Y17" s="88">
         <v>0</v>
       </c>
@@ -2170,7 +2490,7 @@
       </c>
       <c r="AH17" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C17:F17), 1), BIN2HEX(_xlfn.CONCAT(G17:N17), 2), BIN2HEX(_xlfn.CONCAT(O17:V17), 2), BIN2HEX(_xlfn.CONCAT(W17:AD17), 2) )</f>
-        <v>0000108</v>
+        <v>1884008</v>
       </c>
       <c r="AK17" s="14"/>
       <c r="AL17" s="14"/>
@@ -2212,7 +2532,7 @@
       <c r="BV17" s="14"/>
       <c r="BW17" s="14"/>
     </row>
-    <row r="18" spans="1:75" ht="30.95">
+    <row r="18" spans="1:75" ht="31">
       <c r="A18" s="10" t="s">
         <v>35</v>
       </c>
@@ -2246,36 +2566,76 @@
       <c r="AC18" s="77"/>
       <c r="AD18" s="83"/>
     </row>
-    <row r="19" spans="1:75" ht="32.1" customHeight="1">
+    <row r="19" spans="1:75" ht="32.15" customHeight="1">
       <c r="A19" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-      <c r="H19" s="31"/>
-      <c r="I19" s="38"/>
-      <c r="J19" s="38"/>
-      <c r="K19" s="38"/>
-      <c r="L19" s="38"/>
-      <c r="M19" s="49"/>
-      <c r="N19" s="48"/>
+      <c r="C19" s="30">
+        <v>1</v>
+      </c>
+      <c r="D19" s="31">
+        <v>0</v>
+      </c>
+      <c r="E19" s="31">
+        <v>0</v>
+      </c>
+      <c r="F19" s="31">
+        <v>0</v>
+      </c>
+      <c r="G19" s="31">
+        <v>0</v>
+      </c>
+      <c r="H19" s="31">
+        <v>0</v>
+      </c>
+      <c r="I19" s="38">
+        <v>0</v>
+      </c>
+      <c r="J19" s="38">
+        <v>0</v>
+      </c>
+      <c r="K19" s="38">
+        <v>1</v>
+      </c>
+      <c r="L19" s="38">
+        <v>0</v>
+      </c>
+      <c r="M19" s="49">
+        <v>0</v>
+      </c>
+      <c r="N19" s="48">
+        <v>0</v>
+      </c>
       <c r="O19" s="74">
         <v>0</v>
       </c>
       <c r="P19" s="74">
         <v>1</v>
       </c>
-      <c r="Q19" s="48"/>
-      <c r="R19" s="49"/>
-      <c r="S19" s="48"/>
-      <c r="T19" s="48"/>
-      <c r="U19" s="49"/>
-      <c r="V19" s="48"/>
-      <c r="W19" s="65"/>
-      <c r="X19" s="65"/>
+      <c r="Q19" s="48">
+        <v>0</v>
+      </c>
+      <c r="R19" s="49">
+        <v>0</v>
+      </c>
+      <c r="S19" s="48">
+        <v>0</v>
+      </c>
+      <c r="T19" s="48">
+        <v>0</v>
+      </c>
+      <c r="U19" s="49">
+        <v>0</v>
+      </c>
+      <c r="V19" s="48">
+        <v>1</v>
+      </c>
+      <c r="W19" s="65">
+        <v>0</v>
+      </c>
+      <c r="X19" s="65">
+        <v>0</v>
+      </c>
       <c r="Y19" s="77">
         <v>0</v>
       </c>
@@ -2296,39 +2656,79 @@
       </c>
       <c r="AH19" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C19:F19), 1), BIN2HEX(_xlfn.CONCAT(G19:N19), 2), BIN2HEX(_xlfn.CONCAT(O19:V19), 2), BIN2HEX(_xlfn.CONCAT(W19:AD19), 2) )</f>
-        <v>0000113</v>
+        <v>8084113</v>
       </c>
     </row>
     <row r="20" spans="1:75">
       <c r="A20" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="38"/>
-      <c r="J20" s="38"/>
-      <c r="K20" s="38"/>
-      <c r="L20" s="38"/>
-      <c r="M20" s="49"/>
-      <c r="N20" s="48"/>
+      <c r="C20" s="30">
+        <v>0</v>
+      </c>
+      <c r="D20" s="31">
+        <v>1</v>
+      </c>
+      <c r="E20" s="31">
+        <v>0</v>
+      </c>
+      <c r="F20" s="31">
+        <v>0</v>
+      </c>
+      <c r="G20" s="31">
+        <v>0</v>
+      </c>
+      <c r="H20" s="31">
+        <v>0</v>
+      </c>
+      <c r="I20" s="38">
+        <v>0</v>
+      </c>
+      <c r="J20" s="38">
+        <v>0</v>
+      </c>
+      <c r="K20" s="38">
+        <v>0</v>
+      </c>
+      <c r="L20" s="38">
+        <v>0</v>
+      </c>
+      <c r="M20" s="49">
+        <v>0</v>
+      </c>
+      <c r="N20" s="48">
+        <v>0</v>
+      </c>
       <c r="O20" s="74">
         <v>0</v>
       </c>
       <c r="P20" s="74">
         <v>0</v>
       </c>
-      <c r="Q20" s="48"/>
-      <c r="R20" s="49"/>
-      <c r="S20" s="48"/>
-      <c r="T20" s="48"/>
-      <c r="U20" s="49"/>
-      <c r="V20" s="48"/>
-      <c r="W20" s="65"/>
-      <c r="X20" s="65"/>
+      <c r="Q20" s="48">
+        <v>0</v>
+      </c>
+      <c r="R20" s="49">
+        <v>0</v>
+      </c>
+      <c r="S20" s="48">
+        <v>0</v>
+      </c>
+      <c r="T20" s="48">
+        <v>0</v>
+      </c>
+      <c r="U20" s="49">
+        <v>0</v>
+      </c>
+      <c r="V20" s="48">
+        <v>0</v>
+      </c>
+      <c r="W20" s="65">
+        <v>1</v>
+      </c>
+      <c r="X20" s="65">
+        <v>0</v>
+      </c>
       <c r="Y20" s="77">
         <v>1</v>
       </c>
@@ -2349,7 +2749,7 @@
       </c>
       <c r="AH20" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C20:F20), 1), BIN2HEX(_xlfn.CONCAT(G20:N20), 2), BIN2HEX(_xlfn.CONCAT(O20:V20), 2), BIN2HEX(_xlfn.CONCAT(W20:AD20), 2) )</f>
-        <v>0000023</v>
+        <v>40000A3</v>
       </c>
     </row>
     <row r="21" spans="1:75">
@@ -2357,32 +2757,72 @@
         <v>38</v>
       </c>
       <c r="B21" s="8"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
-      <c r="G21" s="29"/>
-      <c r="H21" s="29"/>
-      <c r="I21" s="39"/>
-      <c r="J21" s="39"/>
-      <c r="K21" s="39"/>
-      <c r="L21" s="39"/>
-      <c r="M21" s="58"/>
-      <c r="N21" s="54"/>
+      <c r="C21" s="28">
+        <v>0</v>
+      </c>
+      <c r="D21" s="29">
+        <v>0</v>
+      </c>
+      <c r="E21" s="29">
+        <v>0</v>
+      </c>
+      <c r="F21" s="29">
+        <v>1</v>
+      </c>
+      <c r="G21" s="29">
+        <v>1</v>
+      </c>
+      <c r="H21" s="29">
+        <v>0</v>
+      </c>
+      <c r="I21" s="39">
+        <v>0</v>
+      </c>
+      <c r="J21" s="39">
+        <v>1</v>
+      </c>
+      <c r="K21" s="39">
+        <v>0</v>
+      </c>
+      <c r="L21" s="39">
+        <v>0</v>
+      </c>
+      <c r="M21" s="58">
+        <v>0</v>
+      </c>
+      <c r="N21" s="54">
+        <v>0</v>
+      </c>
       <c r="O21" s="75">
         <v>0</v>
       </c>
       <c r="P21" s="75">
         <v>0</v>
       </c>
-      <c r="Q21" s="54"/>
-      <c r="R21" s="58"/>
-      <c r="S21" s="54"/>
-      <c r="T21" s="54"/>
-      <c r="U21" s="58"/>
-      <c r="V21" s="54"/>
-      <c r="W21" s="66"/>
-      <c r="X21" s="66"/>
+      <c r="Q21" s="54">
+        <v>0</v>
+      </c>
+      <c r="R21" s="58">
+        <v>0</v>
+      </c>
+      <c r="S21" s="54">
+        <v>0</v>
+      </c>
+      <c r="T21" s="54">
+        <v>0</v>
+      </c>
+      <c r="U21" s="58">
+        <v>0</v>
+      </c>
+      <c r="V21" s="54">
+        <v>0</v>
+      </c>
+      <c r="W21" s="66">
+        <v>0</v>
+      </c>
+      <c r="X21" s="66">
+        <v>0</v>
+      </c>
       <c r="Y21" s="88">
         <v>0</v>
       </c>
@@ -2403,10 +2843,10 @@
       </c>
       <c r="AH21" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C21:F21), 1), BIN2HEX(_xlfn.CONCAT(G21:N21), 2), BIN2HEX(_xlfn.CONCAT(O21:V21), 2), BIN2HEX(_xlfn.CONCAT(W21:AD21), 2) )</f>
-        <v>0000008</v>
-      </c>
-    </row>
-    <row r="22" spans="1:75" ht="30.95">
+        <v>1900008</v>
+      </c>
+    </row>
+    <row r="22" spans="1:75" ht="31">
       <c r="A22" s="10" t="s">
         <v>39</v>
       </c>
@@ -2440,36 +2880,76 @@
       <c r="AC22" s="77"/>
       <c r="AD22" s="83"/>
     </row>
-    <row r="23" spans="1:75" ht="32.1" customHeight="1">
+    <row r="23" spans="1:75" ht="32.15" customHeight="1">
       <c r="A23" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
-      <c r="I23" s="38"/>
-      <c r="J23" s="38"/>
-      <c r="K23" s="38"/>
-      <c r="L23" s="38"/>
-      <c r="M23" s="49"/>
-      <c r="N23" s="48"/>
+      <c r="C23" s="30">
+        <v>1</v>
+      </c>
+      <c r="D23" s="31">
+        <v>0</v>
+      </c>
+      <c r="E23" s="31">
+        <v>0</v>
+      </c>
+      <c r="F23" s="31">
+        <v>0</v>
+      </c>
+      <c r="G23" s="31">
+        <v>0</v>
+      </c>
+      <c r="H23" s="31">
+        <v>0</v>
+      </c>
+      <c r="I23" s="38">
+        <v>0</v>
+      </c>
+      <c r="J23" s="38">
+        <v>0</v>
+      </c>
+      <c r="K23" s="38">
+        <v>0</v>
+      </c>
+      <c r="L23" s="38">
+        <v>1</v>
+      </c>
+      <c r="M23" s="49">
+        <v>0</v>
+      </c>
+      <c r="N23" s="48">
+        <v>0</v>
+      </c>
       <c r="O23" s="74">
         <v>0</v>
       </c>
       <c r="P23" s="74">
         <v>0</v>
       </c>
-      <c r="Q23" s="48"/>
-      <c r="R23" s="49"/>
-      <c r="S23" s="48"/>
-      <c r="T23" s="48"/>
-      <c r="U23" s="49"/>
-      <c r="V23" s="48"/>
-      <c r="W23" s="65"/>
-      <c r="X23" s="65"/>
+      <c r="Q23" s="48">
+        <v>0</v>
+      </c>
+      <c r="R23" s="49">
+        <v>1</v>
+      </c>
+      <c r="S23" s="48">
+        <v>1</v>
+      </c>
+      <c r="T23" s="48">
+        <v>1</v>
+      </c>
+      <c r="U23" s="49">
+        <v>0</v>
+      </c>
+      <c r="V23" s="48">
+        <v>0</v>
+      </c>
+      <c r="W23" s="65">
+        <v>0</v>
+      </c>
+      <c r="X23" s="65">
+        <v>0</v>
+      </c>
       <c r="Y23" s="77">
         <v>0</v>
       </c>
@@ -2490,39 +2970,79 @@
       </c>
       <c r="AH23" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C23:F23), 1), BIN2HEX(_xlfn.CONCAT(G23:N23), 2), BIN2HEX(_xlfn.CONCAT(O23:V23), 2), BIN2HEX(_xlfn.CONCAT(W23:AD23), 2) )</f>
-        <v>000001A</v>
+        <v>8041C1A</v>
       </c>
     </row>
     <row r="24" spans="1:75">
       <c r="A24" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="30"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="38"/>
-      <c r="J24" s="38"/>
-      <c r="K24" s="38"/>
-      <c r="L24" s="38"/>
-      <c r="M24" s="49"/>
-      <c r="N24" s="48"/>
+      <c r="C24" s="30">
+        <v>0</v>
+      </c>
+      <c r="D24" s="31">
+        <v>1</v>
+      </c>
+      <c r="E24" s="31">
+        <v>0</v>
+      </c>
+      <c r="F24" s="31">
+        <v>0</v>
+      </c>
+      <c r="G24" s="31">
+        <v>0</v>
+      </c>
+      <c r="H24" s="31">
+        <v>0</v>
+      </c>
+      <c r="I24" s="38">
+        <v>0</v>
+      </c>
+      <c r="J24" s="38">
+        <v>0</v>
+      </c>
+      <c r="K24" s="38">
+        <v>0</v>
+      </c>
+      <c r="L24" s="38">
+        <v>0</v>
+      </c>
+      <c r="M24" s="49">
+        <v>0</v>
+      </c>
+      <c r="N24" s="48">
+        <v>0</v>
+      </c>
       <c r="O24" s="74">
         <v>0</v>
       </c>
       <c r="P24" s="74">
         <v>0</v>
       </c>
-      <c r="Q24" s="48"/>
-      <c r="R24" s="49"/>
-      <c r="S24" s="48"/>
-      <c r="T24" s="48"/>
-      <c r="U24" s="49"/>
-      <c r="V24" s="48"/>
-      <c r="W24" s="65"/>
-      <c r="X24" s="65"/>
+      <c r="Q24" s="48">
+        <v>0</v>
+      </c>
+      <c r="R24" s="49">
+        <v>0</v>
+      </c>
+      <c r="S24" s="48">
+        <v>0</v>
+      </c>
+      <c r="T24" s="48">
+        <v>0</v>
+      </c>
+      <c r="U24" s="49">
+        <v>0</v>
+      </c>
+      <c r="V24" s="48">
+        <v>0</v>
+      </c>
+      <c r="W24" s="65">
+        <v>1</v>
+      </c>
+      <c r="X24" s="65">
+        <v>0</v>
+      </c>
       <c r="Y24" s="77">
         <v>1</v>
       </c>
@@ -2543,39 +3063,79 @@
       </c>
       <c r="AH24" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C24:F24), 1), BIN2HEX(_xlfn.CONCAT(G24:N24), 2), BIN2HEX(_xlfn.CONCAT(O24:V24), 2), BIN2HEX(_xlfn.CONCAT(W24:AD24), 2) )</f>
-        <v>000002A</v>
+        <v>40000AA</v>
       </c>
     </row>
     <row r="25" spans="1:75">
       <c r="A25" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="38"/>
-      <c r="J25" s="38"/>
-      <c r="K25" s="38"/>
-      <c r="L25" s="38"/>
-      <c r="M25" s="49"/>
-      <c r="N25" s="48"/>
+      <c r="C25" s="30">
+        <v>1</v>
+      </c>
+      <c r="D25" s="31">
+        <v>0</v>
+      </c>
+      <c r="E25" s="31">
+        <v>0</v>
+      </c>
+      <c r="F25" s="31">
+        <v>0</v>
+      </c>
+      <c r="G25" s="31">
+        <v>0</v>
+      </c>
+      <c r="H25" s="31">
+        <v>0</v>
+      </c>
+      <c r="I25" s="38">
+        <v>0</v>
+      </c>
+      <c r="J25" s="38">
+        <v>1</v>
+      </c>
+      <c r="K25" s="38">
+        <v>0</v>
+      </c>
+      <c r="L25" s="38">
+        <v>0</v>
+      </c>
+      <c r="M25" s="49">
+        <v>0</v>
+      </c>
+      <c r="N25" s="48">
+        <v>0</v>
+      </c>
       <c r="O25" s="74">
         <v>0</v>
       </c>
       <c r="P25" s="74">
         <v>0</v>
       </c>
-      <c r="Q25" s="48"/>
-      <c r="R25" s="49"/>
-      <c r="S25" s="48"/>
-      <c r="T25" s="48"/>
-      <c r="U25" s="49"/>
-      <c r="V25" s="48"/>
-      <c r="W25" s="65"/>
-      <c r="X25" s="65"/>
+      <c r="Q25" s="48">
+        <v>0</v>
+      </c>
+      <c r="R25" s="49">
+        <v>0</v>
+      </c>
+      <c r="S25" s="48">
+        <v>0</v>
+      </c>
+      <c r="T25" s="48">
+        <v>0</v>
+      </c>
+      <c r="U25" s="49">
+        <v>0</v>
+      </c>
+      <c r="V25" s="48">
+        <v>0</v>
+      </c>
+      <c r="W25" s="65">
+        <v>0</v>
+      </c>
+      <c r="X25" s="65">
+        <v>0</v>
+      </c>
       <c r="Y25" s="77">
         <v>1</v>
       </c>
@@ -2596,39 +3156,79 @@
       </c>
       <c r="AH25" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C25:F25), 1), BIN2HEX(_xlfn.CONCAT(G25:N25), 2), BIN2HEX(_xlfn.CONCAT(O25:V25), 2), BIN2HEX(_xlfn.CONCAT(W25:AD25), 2) )</f>
-        <v>000003A</v>
+        <v>810003A</v>
       </c>
     </row>
     <row r="26" spans="1:75">
       <c r="A26" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="30"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31"/>
-      <c r="I26" s="38"/>
-      <c r="J26" s="38"/>
-      <c r="K26" s="38"/>
-      <c r="L26" s="38"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="48"/>
+      <c r="C26" s="30">
+        <v>0</v>
+      </c>
+      <c r="D26" s="31">
+        <v>1</v>
+      </c>
+      <c r="E26" s="31">
+        <v>0</v>
+      </c>
+      <c r="F26" s="31">
+        <v>0</v>
+      </c>
+      <c r="G26" s="31">
+        <v>0</v>
+      </c>
+      <c r="H26" s="31">
+        <v>0</v>
+      </c>
+      <c r="I26" s="38">
+        <v>1</v>
+      </c>
+      <c r="J26" s="38">
+        <v>0</v>
+      </c>
+      <c r="K26" s="38">
+        <v>0</v>
+      </c>
+      <c r="L26" s="38">
+        <v>0</v>
+      </c>
+      <c r="M26" s="49">
+        <v>0</v>
+      </c>
+      <c r="N26" s="48">
+        <v>0</v>
+      </c>
       <c r="O26" s="74">
         <v>0</v>
       </c>
       <c r="P26" s="74">
         <v>0</v>
       </c>
-      <c r="Q26" s="48"/>
-      <c r="R26" s="49"/>
-      <c r="S26" s="48"/>
-      <c r="T26" s="48"/>
-      <c r="U26" s="49"/>
-      <c r="V26" s="48"/>
-      <c r="W26" s="65"/>
-      <c r="X26" s="65"/>
+      <c r="Q26" s="48">
+        <v>0</v>
+      </c>
+      <c r="R26" s="49">
+        <v>0</v>
+      </c>
+      <c r="S26" s="48">
+        <v>0</v>
+      </c>
+      <c r="T26" s="48">
+        <v>0</v>
+      </c>
+      <c r="U26" s="49">
+        <v>0</v>
+      </c>
+      <c r="V26" s="48">
+        <v>0</v>
+      </c>
+      <c r="W26" s="65">
+        <v>0</v>
+      </c>
+      <c r="X26" s="65">
+        <v>0</v>
+      </c>
       <c r="Y26" s="77">
         <v>0</v>
       </c>
@@ -2649,7 +3249,7 @@
       </c>
       <c r="AH26" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C26:F26), 1), BIN2HEX(_xlfn.CONCAT(G26:N26), 2), BIN2HEX(_xlfn.CONCAT(O26:V26), 2), BIN2HEX(_xlfn.CONCAT(W26:AD26), 2) )</f>
-        <v>000001D</v>
+        <v>420001D</v>
       </c>
     </row>
     <row r="27" spans="1:75">
@@ -2657,32 +3257,72 @@
         <v>44</v>
       </c>
       <c r="B27" s="8"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="39"/>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="39"/>
-      <c r="M27" s="58"/>
-      <c r="N27" s="54"/>
+      <c r="C27" s="28">
+        <v>0</v>
+      </c>
+      <c r="D27" s="29">
+        <v>0</v>
+      </c>
+      <c r="E27" s="29">
+        <v>0</v>
+      </c>
+      <c r="F27" s="29">
+        <v>0</v>
+      </c>
+      <c r="G27" s="29">
+        <v>0</v>
+      </c>
+      <c r="H27" s="29">
+        <v>0</v>
+      </c>
+      <c r="I27" s="39">
+        <v>0</v>
+      </c>
+      <c r="J27" s="39">
+        <v>0</v>
+      </c>
+      <c r="K27" s="39">
+        <v>0</v>
+      </c>
+      <c r="L27" s="39">
+        <v>0</v>
+      </c>
+      <c r="M27" s="58">
+        <v>0</v>
+      </c>
+      <c r="N27" s="54">
+        <v>0</v>
+      </c>
       <c r="O27" s="75">
         <v>0</v>
       </c>
       <c r="P27" s="75">
         <v>0</v>
       </c>
-      <c r="Q27" s="54"/>
-      <c r="R27" s="58"/>
-      <c r="S27" s="54"/>
-      <c r="T27" s="54"/>
-      <c r="U27" s="58"/>
-      <c r="V27" s="54"/>
-      <c r="W27" s="66"/>
-      <c r="X27" s="66"/>
+      <c r="Q27" s="54">
+        <v>0</v>
+      </c>
+      <c r="R27" s="58">
+        <v>0</v>
+      </c>
+      <c r="S27" s="54">
+        <v>0</v>
+      </c>
+      <c r="T27" s="54">
+        <v>0</v>
+      </c>
+      <c r="U27" s="58">
+        <v>0</v>
+      </c>
+      <c r="V27" s="54">
+        <v>0</v>
+      </c>
+      <c r="W27" s="66">
+        <v>1</v>
+      </c>
+      <c r="X27" s="66">
+        <v>1</v>
+      </c>
       <c r="Y27" s="88">
         <v>0</v>
       </c>
@@ -2703,10 +3343,10 @@
       </c>
       <c r="AH27" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C27:F27), 1), BIN2HEX(_xlfn.CONCAT(G27:N27), 2), BIN2HEX(_xlfn.CONCAT(O27:V27), 2), BIN2HEX(_xlfn.CONCAT(W27:AD27), 2) )</f>
-        <v>0000008</v>
-      </c>
-    </row>
-    <row r="28" spans="1:75" ht="30.95">
+        <v>00000C8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:75" ht="31">
       <c r="A28" s="10" t="s">
         <v>45</v>
       </c>
@@ -2744,32 +3384,72 @@
       <c r="A29" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="31"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="38"/>
-      <c r="J29" s="38"/>
-      <c r="K29" s="38"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="49"/>
-      <c r="N29" s="48"/>
+      <c r="C29" s="30">
+        <v>0</v>
+      </c>
+      <c r="D29" s="31">
+        <v>0</v>
+      </c>
+      <c r="E29" s="31">
+        <v>0</v>
+      </c>
+      <c r="F29" s="31">
+        <v>1</v>
+      </c>
+      <c r="G29" s="31">
+        <v>0</v>
+      </c>
+      <c r="H29" s="31">
+        <v>0</v>
+      </c>
+      <c r="I29" s="38">
+        <v>0</v>
+      </c>
+      <c r="J29" s="38">
+        <v>0</v>
+      </c>
+      <c r="K29" s="38">
+        <v>0</v>
+      </c>
+      <c r="L29" s="38">
+        <v>1</v>
+      </c>
+      <c r="M29" s="49">
+        <v>0</v>
+      </c>
+      <c r="N29" s="48">
+        <v>0</v>
+      </c>
       <c r="O29" s="74">
         <v>0</v>
       </c>
       <c r="P29" s="74">
         <v>0</v>
       </c>
-      <c r="Q29" s="48"/>
-      <c r="R29" s="49"/>
-      <c r="S29" s="48"/>
-      <c r="T29" s="48"/>
-      <c r="U29" s="49"/>
-      <c r="V29" s="48"/>
-      <c r="W29" s="65"/>
-      <c r="X29" s="65"/>
+      <c r="Q29" s="48">
+        <v>1</v>
+      </c>
+      <c r="R29" s="49">
+        <v>0</v>
+      </c>
+      <c r="S29" s="48">
+        <v>0</v>
+      </c>
+      <c r="T29" s="48">
+        <v>0</v>
+      </c>
+      <c r="U29" s="49">
+        <v>0</v>
+      </c>
+      <c r="V29" s="48">
+        <v>0</v>
+      </c>
+      <c r="W29" s="65">
+        <v>0</v>
+      </c>
+      <c r="X29" s="65">
+        <v>0</v>
+      </c>
       <c r="Y29" s="77">
         <v>0</v>
       </c>
@@ -2790,39 +3470,79 @@
       </c>
       <c r="AH29" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C29:F29), 1), BIN2HEX(_xlfn.CONCAT(G29:N29), 2), BIN2HEX(_xlfn.CONCAT(O29:V29), 2), BIN2HEX(_xlfn.CONCAT(W29:AD29), 2) )</f>
-        <v>000001F</v>
-      </c>
-    </row>
-    <row r="30" spans="1:75" ht="14.45" customHeight="1">
+        <v>104201F</v>
+      </c>
+    </row>
+    <row r="30" spans="1:75" ht="14.5" customHeight="1">
       <c r="A30" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="30"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="31"/>
-      <c r="H30" s="31"/>
-      <c r="I30" s="38"/>
-      <c r="J30" s="38"/>
-      <c r="K30" s="38"/>
-      <c r="L30" s="38"/>
-      <c r="M30" s="49"/>
-      <c r="N30" s="48"/>
+      <c r="C30" s="30">
+        <v>0</v>
+      </c>
+      <c r="D30" s="31">
+        <v>0</v>
+      </c>
+      <c r="E30" s="31">
+        <v>0</v>
+      </c>
+      <c r="F30" s="31">
+        <v>1</v>
+      </c>
+      <c r="G30" s="31">
+        <v>0</v>
+      </c>
+      <c r="H30" s="31">
+        <v>0</v>
+      </c>
+      <c r="I30" s="38">
+        <v>0</v>
+      </c>
+      <c r="J30" s="38">
+        <v>0</v>
+      </c>
+      <c r="K30" s="38">
+        <v>1</v>
+      </c>
+      <c r="L30" s="38">
+        <v>0</v>
+      </c>
+      <c r="M30" s="49">
+        <v>0</v>
+      </c>
+      <c r="N30" s="48">
+        <v>0</v>
+      </c>
       <c r="O30" s="74">
         <v>0</v>
       </c>
       <c r="P30" s="74">
         <v>1</v>
       </c>
-      <c r="Q30" s="48"/>
-      <c r="R30" s="49"/>
-      <c r="S30" s="48"/>
-      <c r="T30" s="48"/>
-      <c r="U30" s="49"/>
-      <c r="V30" s="48"/>
-      <c r="W30" s="65"/>
-      <c r="X30" s="65"/>
+      <c r="Q30" s="48">
+        <v>0</v>
+      </c>
+      <c r="R30" s="49">
+        <v>0</v>
+      </c>
+      <c r="S30" s="48">
+        <v>0</v>
+      </c>
+      <c r="T30" s="48">
+        <v>0</v>
+      </c>
+      <c r="U30" s="49">
+        <v>0</v>
+      </c>
+      <c r="V30" s="48">
+        <v>1</v>
+      </c>
+      <c r="W30" s="65">
+        <v>0</v>
+      </c>
+      <c r="X30" s="65">
+        <v>0</v>
+      </c>
       <c r="Y30" s="77">
         <v>0</v>
       </c>
@@ -2843,7 +3563,7 @@
       </c>
       <c r="AH30" t="str">
         <f>_xlfn.CONCAT(BIN2HEX(_xlfn.CONCAT(C30:F30), 1), BIN2HEX(_xlfn.CONCAT(G30:N30), 2), BIN2HEX(_xlfn.CONCAT(O30:V30), 2), BIN2HEX(_xlfn.CONCAT(W30:AD30), 2) )</f>
-        <v>0000108</v>
+        <v>1084108</v>
       </c>
     </row>
     <row r="31" spans="1:75">
@@ -2878,13 +3598,13 @@
       <c r="AC31" s="77"/>
       <c r="AD31" s="77"/>
     </row>
-    <row r="38" ht="32.1" customHeight="1"/>
-    <row r="43" ht="32.1" customHeight="1"/>
-    <row r="46" ht="32.1" customHeight="1"/>
-    <row r="49" ht="32.1" customHeight="1"/>
-    <row r="54" ht="14.1" customHeight="1"/>
-    <row r="59" ht="32.1" customHeight="1"/>
-    <row r="66" ht="32.1" customHeight="1"/>
+    <row r="38" ht="32.15" customHeight="1"/>
+    <row r="43" ht="32.15" customHeight="1"/>
+    <row r="46" ht="32.15" customHeight="1"/>
+    <row r="49" ht="32.15" customHeight="1"/>
+    <row r="54" ht="14.15" customHeight="1"/>
+    <row r="59" ht="32.15" customHeight="1"/>
+    <row r="66" ht="32.15" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2894,10 +3614,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G64"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultColWidth="11.08203125" defaultRowHeight="15.5"/>
   <cols>
     <col min="3" max="3" width="15.5" customWidth="1"/>
-    <col min="6" max="6" width="10.625" customWidth="1"/>
+    <col min="6" max="6" width="10.58203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2931,7 +3651,7 @@
       </c>
       <c r="D2" s="16" t="str">
         <f>microcode!AH4</f>
-        <v>0000008</v>
+        <v>1843708</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2962,7 +3682,7 @@
       </c>
       <c r="D4" s="20" t="str">
         <f>microcode!AH19</f>
-        <v>0000113</v>
+        <v>8084113</v>
       </c>
       <c r="E4" t="s">
         <v>53</v>
@@ -3002,14 +3722,14 @@
       </c>
       <c r="D6" t="str">
         <f>microcode!AH29</f>
-        <v>000001F</v>
+        <v>104201F</v>
       </c>
       <c r="E6" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="16" t="str">
         <f>microcode!AH9</f>
-        <v>0000008</v>
+        <v>0520008</v>
       </c>
       <c r="G6" s="15" t="s">
         <v>57</v>
@@ -3028,14 +3748,14 @@
       </c>
       <c r="D7" t="str">
         <f>microcode!AH15</f>
-        <v>0000116</v>
+        <v>1884016</v>
       </c>
       <c r="E7" t="s">
         <v>53</v>
       </c>
       <c r="F7" s="16" t="str">
         <f>microcode!AH15</f>
-        <v>0000116</v>
+        <v>1884016</v>
       </c>
       <c r="G7" s="15" t="s">
         <v>58</v>
@@ -3054,7 +3774,7 @@
       </c>
       <c r="D8" s="20" t="str">
         <f>microcode!AH7</f>
-        <v>0000017</v>
+        <v>8041417</v>
       </c>
       <c r="E8" t="s">
         <v>53</v>
@@ -3109,7 +3829,7 @@
       </c>
       <c r="D11" t="str">
         <f>microcode!AH23</f>
-        <v>000001A</v>
+        <v>8041C1A</v>
       </c>
       <c r="E11" t="s">
         <v>53</v>
@@ -3149,7 +3869,7 @@
       </c>
       <c r="D13" s="16" t="str">
         <f>microcode!AH12</f>
-        <v>0000008</v>
+        <v>0461C08</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -3258,13 +3978,13 @@
       </c>
       <c r="D20" s="20" t="str">
         <f>microcode!AH20</f>
-        <v>0000023</v>
+        <v>40000A3</v>
       </c>
       <c r="E20" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="17.100000000000001">
+    <row r="21" spans="1:7" ht="17">
       <c r="A21" s="15">
         <v>20</v>
       </c>
@@ -3314,7 +4034,7 @@
       </c>
       <c r="D23" s="16" t="str">
         <f>microcode!AH16</f>
-        <v>0000126</v>
+        <v>1884026</v>
       </c>
       <c r="E23" t="s">
         <v>53</v>
@@ -3333,7 +4053,7 @@
       </c>
       <c r="D24" s="20" t="str">
         <f>microcode!AH8</f>
-        <v>0000027</v>
+        <v>40000A7</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
@@ -3388,7 +4108,7 @@
       </c>
       <c r="D27" t="str">
         <f>microcode!AH24</f>
-        <v>000002A</v>
+        <v>40000AA</v>
       </c>
       <c r="E27" t="s">
         <v>53</v>
@@ -3443,7 +4163,7 @@
       </c>
       <c r="D30" t="str">
         <f>microcode!AH27</f>
-        <v>0000008</v>
+        <v>00000C8</v>
       </c>
       <c r="E30" t="s">
         <v>53</v>
@@ -3483,7 +4203,7 @@
       </c>
       <c r="D32" s="16" t="str">
         <f>microcode!AH30</f>
-        <v>0000108</v>
+        <v>1084108</v>
       </c>
       <c r="E32" t="s">
         <v>53</v>
@@ -3547,7 +4267,7 @@
       </c>
       <c r="D36" s="20" t="str">
         <f>microcode!AH21</f>
-        <v>0000008</v>
+        <v>1900008</v>
       </c>
       <c r="E36" t="s">
         <v>53</v>
@@ -3596,7 +4316,7 @@
       </c>
       <c r="D39" s="16" t="str">
         <f>microcode!AH17</f>
-        <v>0000108</v>
+        <v>1884008</v>
       </c>
       <c r="E39" t="s">
         <v>53</v>
@@ -3615,7 +4335,7 @@
       </c>
       <c r="D40" t="str">
         <f>microcode!AH9</f>
-        <v>0000008</v>
+        <v>0520008</v>
       </c>
       <c r="E40" t="s">
         <v>53</v>
@@ -3670,7 +4390,7 @@
       </c>
       <c r="D43" t="str">
         <f>microcode!AH25</f>
-        <v>000003A</v>
+        <v>810003A</v>
       </c>
       <c r="E43" t="s">
         <v>53</v>
@@ -3920,7 +4640,7 @@
       </c>
       <c r="D59" t="str">
         <f>microcode!AH26</f>
-        <v>000001D</v>
+        <v>420001D</v>
       </c>
       <c r="E59" t="s">
         <v>53</v>

</xml_diff>